<commit_message>
pendiente actualizar codigo de los graficos y revisar resultados
</commit_message>
<xml_diff>
--- a/data/Escenarios_Gx/elmo_data.xlsx
+++ b/data/Escenarios_Gx/elmo_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\Escenarios_Gx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Agustin\Desktop\Elmo_infrastructure_NP\data\Escenarios_Gx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE1228C2-4E65-4EDD-AEF5-8BAA87B9EE58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BD8C492-F28E-43D1-8014-750B924F853B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LHD" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="200">
   <si>
     <t>id</t>
   </si>
@@ -530,18 +530,6 @@
     <t>station_name</t>
   </si>
   <si>
-    <t>station_cost</t>
-  </si>
-  <si>
-    <t>distance_to_dn</t>
-  </si>
-  <si>
-    <t>max_chargers</t>
-  </si>
-  <si>
-    <t>man_time</t>
-  </si>
-  <si>
     <t>USD</t>
   </si>
   <si>
@@ -572,9 +560,6 @@
     <t>p_max_ssee</t>
   </si>
   <si>
-    <t>max_batteries</t>
-  </si>
-  <si>
     <t>battery_cost</t>
   </si>
   <si>
@@ -630,6 +615,30 @@
   </si>
   <si>
     <t>Bess</t>
+  </si>
+  <si>
+    <t>c_fixed</t>
+  </si>
+  <si>
+    <t>c_bays</t>
+  </si>
+  <si>
+    <t>c_crane</t>
+  </si>
+  <si>
+    <t>c_charger_space</t>
+  </si>
+  <si>
+    <t>c_battery_space</t>
+  </si>
+  <si>
+    <t>max_bays</t>
+  </si>
+  <si>
+    <t>max_batteries_per_bay</t>
+  </si>
+  <si>
+    <t>max_chargers_per_bay</t>
   </si>
 </sst>
 </file>
@@ -1501,36 +1510,36 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:AE9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" style="23" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" style="23" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.28515625" style="23" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5703125" style="23" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.42578125" style="23" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.109375" style="23" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" style="23" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5546875" style="23" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.44140625" style="23" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="7" style="23" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5703125" style="23" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.7109375" style="24" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.5546875" style="23" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.6640625" style="24" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.109375" style="23" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="15" style="23" customWidth="1"/>
-    <col min="16" max="16" width="17.140625" style="23" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.5703125" style="24" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.109375" style="23" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.5546875" style="24" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="18" style="24" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="20.85546875" style="24" bestFit="1" customWidth="1"/>
-    <col min="20" max="23" width="20.85546875" style="24" customWidth="1"/>
-    <col min="24" max="24" width="18.42578125" style="24" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="20.140625" style="24" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="13.5703125" style="24" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.28515625" style="24" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="20.88671875" style="24" bestFit="1" customWidth="1"/>
+    <col min="20" max="23" width="20.88671875" style="24" customWidth="1"/>
+    <col min="24" max="24" width="18.44140625" style="24" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="20.109375" style="24" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="13.5546875" style="24" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.33203125" style="24" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -1622,10 +1631,10 @@
         <v>62</v>
       </c>
       <c r="AE1" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="2" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="2" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="30" t="s">
         <v>3</v>
       </c>
@@ -1714,13 +1723,13 @@
         <v>37</v>
       </c>
       <c r="AD2" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="AE2" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="3" spans="1:31" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3" spans="1:31" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="31">
         <v>1</v>
       </c>
@@ -1731,7 +1740,7 @@
         <v>161</v>
       </c>
       <c r="D3" s="29" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="E3" s="21" t="s">
         <v>52</v>
@@ -1815,7 +1824,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:31" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="31">
         <v>2</v>
       </c>
@@ -1826,7 +1835,7 @@
         <v>161</v>
       </c>
       <c r="D4" s="29" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="E4" s="21" t="s">
         <v>52</v>
@@ -1910,7 +1919,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:31" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="31">
         <v>3</v>
       </c>
@@ -1921,7 +1930,7 @@
         <v>161</v>
       </c>
       <c r="D5" s="29" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="E5" s="21" t="s">
         <v>52</v>
@@ -2005,7 +2014,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:31" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="31">
         <v>4</v>
       </c>
@@ -2016,7 +2025,7 @@
         <v>161</v>
       </c>
       <c r="D6" s="29" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="E6" s="21" t="s">
         <v>52</v>
@@ -2101,9 +2110,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="1:31" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2112,88 +2121,106 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC93900-5A86-4519-AB89-460E8AC441EE}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="B1" t="s">
-        <v>162</v>
+        <v>192</v>
       </c>
       <c r="C1" t="s">
+        <v>193</v>
+      </c>
+      <c r="D1" t="s">
+        <v>194</v>
+      </c>
+      <c r="E1" t="s">
+        <v>195</v>
+      </c>
+      <c r="F1" t="s">
+        <v>196</v>
+      </c>
+      <c r="G1" t="s">
+        <v>197</v>
+      </c>
+      <c r="H1" t="s">
+        <v>198</v>
+      </c>
+      <c r="I1" t="s">
+        <v>199</v>
+      </c>
+      <c r="J1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
         <v>163</v>
       </c>
-      <c r="D1" t="s">
-        <v>164</v>
-      </c>
-      <c r="E1" t="s">
-        <v>165</v>
-      </c>
-      <c r="F1" t="s">
-        <v>166</v>
-      </c>
-      <c r="G1" t="s">
-        <v>177</v>
-      </c>
-      <c r="H1" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
       <c r="C2" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>163</v>
       </c>
       <c r="E2" t="s">
-        <v>51</v>
+        <v>163</v>
       </c>
       <c r="F2" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="G2" t="s">
         <v>51</v>
       </c>
       <c r="H2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I2" t="s">
+        <v>51</v>
+      </c>
+      <c r="J2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>169</v>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B3">
+        <v>35722</v>
       </c>
       <c r="C3">
-        <v>215756</v>
+        <v>38221</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>16752</v>
       </c>
       <c r="E3">
-        <v>4</v>
+        <v>5733</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>4389</v>
       </c>
       <c r="G3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+      <c r="J3">
         <v>1500</v>
       </c>
     </row>
@@ -2206,35 +2233,35 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA5C58D2-31A1-4CA6-99E5-3102447D41CF}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C1" t="s">
+        <v>167</v>
+      </c>
+      <c r="D1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F1" t="s">
         <v>170</v>
       </c>
-      <c r="C1" t="s">
-        <v>171</v>
-      </c>
-      <c r="D1" t="s">
-        <v>172</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>173</v>
-      </c>
-      <c r="F1" t="s">
-        <v>174</v>
-      </c>
-      <c r="G1" t="s">
-        <v>178</v>
       </c>
       <c r="H1" s="13" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2242,7 +2269,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D2" t="s">
         <v>34</v>
@@ -2254,18 +2281,18 @@
         <v>34</v>
       </c>
       <c r="G2" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="H2" s="33" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C3">
         <v>42071</v>
@@ -2297,17 +2324,17 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:H152"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" style="49" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" style="11" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.42578125" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="29.140625" style="69" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" style="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" style="49" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" style="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.44140625" style="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="29.109375" style="69" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5546875" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="50" t="s">
         <v>0</v>
       </c>
@@ -2333,7 +2360,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="51" t="s">
         <v>3</v>
       </c>
@@ -2359,7 +2386,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="52">
         <v>0</v>
       </c>
@@ -2385,7 +2412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="53">
         <v>1</v>
       </c>
@@ -2411,7 +2438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="53">
         <v>2</v>
       </c>
@@ -2437,7 +2464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="52">
         <v>3</v>
       </c>
@@ -2463,7 +2490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="53">
         <v>4</v>
       </c>
@@ -2489,7 +2516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="53">
         <v>5</v>
       </c>
@@ -2515,7 +2542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="52">
         <v>6</v>
       </c>
@@ -2541,7 +2568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="53">
         <v>7</v>
       </c>
@@ -2567,7 +2594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="53">
         <v>8</v>
       </c>
@@ -2593,7 +2620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="52">
         <v>9</v>
       </c>
@@ -2619,7 +2646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="53">
         <v>10</v>
       </c>
@@ -2645,7 +2672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="53">
         <v>11</v>
       </c>
@@ -2671,7 +2698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="53">
         <v>12</v>
       </c>
@@ -2697,7 +2724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="52">
         <v>13</v>
       </c>
@@ -2723,7 +2750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="53">
         <v>14</v>
       </c>
@@ -2749,7 +2776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="53">
         <v>15</v>
       </c>
@@ -2775,7 +2802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="52">
         <v>16</v>
       </c>
@@ -2801,7 +2828,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="53">
         <v>17</v>
       </c>
@@ -2827,7 +2854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="53">
         <v>18</v>
       </c>
@@ -2853,7 +2880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="52">
         <v>19</v>
       </c>
@@ -2879,7 +2906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="53">
         <v>20</v>
       </c>
@@ -2905,7 +2932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="53">
         <v>21</v>
       </c>
@@ -2931,7 +2958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="53">
         <v>22</v>
       </c>
@@ -2957,7 +2984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="52">
         <v>23</v>
       </c>
@@ -2983,7 +3010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="53">
         <v>24</v>
       </c>
@@ -3009,7 +3036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="52">
         <v>25</v>
       </c>
@@ -3035,7 +3062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="53">
         <v>26</v>
       </c>
@@ -3061,7 +3088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="53">
         <v>27</v>
       </c>
@@ -3087,7 +3114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="52">
         <v>28</v>
       </c>
@@ -3113,7 +3140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="53">
         <v>29</v>
       </c>
@@ -3139,7 +3166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="53">
         <v>30</v>
       </c>
@@ -3165,7 +3192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="52">
         <v>31</v>
       </c>
@@ -3191,7 +3218,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="53">
         <v>32</v>
       </c>
@@ -3217,7 +3244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="53">
         <v>33</v>
       </c>
@@ -3243,7 +3270,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="52">
         <v>34</v>
       </c>
@@ -3269,7 +3296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="53">
         <v>35</v>
       </c>
@@ -3295,7 +3322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="53">
         <v>36</v>
       </c>
@@ -3321,7 +3348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="53">
         <v>37</v>
       </c>
@@ -3347,7 +3374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="52">
         <v>38</v>
       </c>
@@ -3373,7 +3400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="53">
         <v>39</v>
       </c>
@@ -3399,7 +3426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="53">
         <v>40</v>
       </c>
@@ -3425,7 +3452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" s="53">
         <v>41</v>
       </c>
@@ -3451,7 +3478,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="53">
         <v>42</v>
       </c>
@@ -3477,7 +3504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" s="53">
         <v>43</v>
       </c>
@@ -3503,7 +3530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="53">
         <v>44</v>
       </c>
@@ -3529,7 +3556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" s="53">
         <v>45</v>
       </c>
@@ -3555,7 +3582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" s="53">
         <v>46</v>
       </c>
@@ -3581,7 +3608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="53">
         <v>47</v>
       </c>
@@ -3607,7 +3634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" s="53">
         <v>48</v>
       </c>
@@ -3633,7 +3660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" s="53">
         <v>49</v>
       </c>
@@ -3659,7 +3686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53" s="53">
         <v>50</v>
       </c>
@@ -3685,7 +3712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" s="53">
         <v>51</v>
       </c>
@@ -3711,7 +3738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" s="53">
         <v>52</v>
       </c>
@@ -3737,7 +3764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" s="53">
         <v>53</v>
       </c>
@@ -3763,7 +3790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" s="53">
         <v>54</v>
       </c>
@@ -3789,7 +3816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" s="53">
         <v>55</v>
       </c>
@@ -3815,7 +3842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59" s="53">
         <v>56</v>
       </c>
@@ -3841,7 +3868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60" s="53">
         <v>57</v>
       </c>
@@ -3867,7 +3894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61" s="53">
         <v>58</v>
       </c>
@@ -3893,7 +3920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" s="53">
         <v>59</v>
       </c>
@@ -3919,7 +3946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63" s="53">
         <v>60</v>
       </c>
@@ -3945,7 +3972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64" s="53">
         <v>61</v>
       </c>
@@ -3971,7 +3998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="53">
         <v>62</v>
       </c>
@@ -3997,7 +4024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66" s="53">
         <v>63</v>
       </c>
@@ -4023,7 +4050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" s="53">
         <v>64</v>
       </c>
@@ -4049,7 +4076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" s="53">
         <v>65</v>
       </c>
@@ -4075,7 +4102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="53">
         <v>66</v>
       </c>
@@ -4101,7 +4128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" s="53">
         <v>67</v>
       </c>
@@ -4127,7 +4154,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" s="53">
         <v>68</v>
       </c>
@@ -4153,7 +4180,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" s="53">
         <v>69</v>
       </c>
@@ -4179,7 +4206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" s="53">
         <v>70</v>
       </c>
@@ -4205,7 +4232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" s="53">
         <v>71</v>
       </c>
@@ -4231,7 +4258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="53">
         <v>72</v>
       </c>
@@ -4257,7 +4284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" s="53">
         <v>73</v>
       </c>
@@ -4283,7 +4310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="53">
         <v>74</v>
       </c>
@@ -4309,7 +4336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" s="53">
         <v>75</v>
       </c>
@@ -4335,7 +4362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" s="53">
         <v>76</v>
       </c>
@@ -4361,7 +4388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="53">
         <v>77</v>
       </c>
@@ -4387,7 +4414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A81" s="53">
         <v>78</v>
       </c>
@@ -4413,7 +4440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A82" s="53">
         <v>79</v>
       </c>
@@ -4439,7 +4466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A83" s="53">
         <v>80</v>
       </c>
@@ -4465,7 +4492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A84" s="53">
         <v>81</v>
       </c>
@@ -4491,7 +4518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A85" s="53">
         <v>82</v>
       </c>
@@ -4517,7 +4544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A86" s="53">
         <v>83</v>
       </c>
@@ -4543,7 +4570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A87" s="53">
         <v>84</v>
       </c>
@@ -4569,7 +4596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A88" s="53">
         <v>85</v>
       </c>
@@ -4595,7 +4622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A89" s="53">
         <v>86</v>
       </c>
@@ -4621,7 +4648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A90" s="53">
         <v>87</v>
       </c>
@@ -4647,7 +4674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A91" s="53">
         <v>88</v>
       </c>
@@ -4673,7 +4700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A92" s="53">
         <v>89</v>
       </c>
@@ -4699,7 +4726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A93" s="53">
         <v>90</v>
       </c>
@@ -4725,7 +4752,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A94" s="53">
         <v>91</v>
       </c>
@@ -4751,7 +4778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A95" s="53">
         <v>92</v>
       </c>
@@ -4777,7 +4804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A96" s="53">
         <v>93</v>
       </c>
@@ -4803,10 +4830,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A97" s="53"/>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A98" s="54"/>
       <c r="B98" s="64"/>
       <c r="C98" s="61"/>
@@ -4814,7 +4841,7 @@
       <c r="G98" s="43"/>
       <c r="H98" s="44"/>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A99" s="55"/>
       <c r="B99" s="64"/>
       <c r="C99" s="62"/>
@@ -4822,7 +4849,7 @@
       <c r="G99" s="37"/>
       <c r="H99" s="8"/>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A100" s="56"/>
       <c r="B100" s="64"/>
       <c r="C100" s="62"/>
@@ -4830,7 +4857,7 @@
       <c r="G100" s="37"/>
       <c r="H100" s="8"/>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A101" s="57"/>
       <c r="B101" s="64"/>
       <c r="C101" s="62"/>
@@ -4838,7 +4865,7 @@
       <c r="G101" s="37"/>
       <c r="H101" s="8"/>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A102" s="57"/>
       <c r="B102" s="64"/>
       <c r="C102" s="62"/>
@@ -4846,7 +4873,7 @@
       <c r="G102" s="37"/>
       <c r="H102" s="8"/>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A103" s="57"/>
       <c r="B103" s="64"/>
       <c r="C103" s="62"/>
@@ -4854,7 +4881,7 @@
       <c r="G103" s="37"/>
       <c r="H103" s="8"/>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A104" s="55"/>
       <c r="B104" s="64"/>
       <c r="C104" s="62"/>
@@ -4862,7 +4889,7 @@
       <c r="G104" s="37"/>
       <c r="H104" s="8"/>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A105" s="56"/>
       <c r="B105" s="64"/>
       <c r="C105" s="62"/>
@@ -4870,7 +4897,7 @@
       <c r="G105" s="37"/>
       <c r="H105" s="8"/>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A106" s="57"/>
       <c r="B106" s="64"/>
       <c r="C106" s="62"/>
@@ -4878,7 +4905,7 @@
       <c r="G106" s="37"/>
       <c r="H106" s="8"/>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A107" s="57"/>
       <c r="B107" s="64"/>
       <c r="C107" s="62"/>
@@ -4886,7 +4913,7 @@
       <c r="G107" s="37"/>
       <c r="H107" s="8"/>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A108" s="57"/>
       <c r="B108" s="64"/>
       <c r="C108" s="62"/>
@@ -4894,7 +4921,7 @@
       <c r="G108" s="37"/>
       <c r="H108" s="8"/>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A109" s="55"/>
       <c r="B109" s="64"/>
       <c r="C109" s="62"/>
@@ -4902,7 +4929,7 @@
       <c r="G109" s="37"/>
       <c r="H109" s="8"/>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A110" s="56"/>
       <c r="B110" s="64"/>
       <c r="C110" s="62"/>
@@ -4910,7 +4937,7 @@
       <c r="G110" s="37"/>
       <c r="H110" s="8"/>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A111" s="57"/>
       <c r="B111" s="64"/>
       <c r="C111" s="62"/>
@@ -4918,7 +4945,7 @@
       <c r="G111" s="37"/>
       <c r="H111" s="8"/>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A112" s="57"/>
       <c r="B112" s="64"/>
       <c r="C112" s="62"/>
@@ -4926,7 +4953,7 @@
       <c r="G112" s="37"/>
       <c r="H112" s="8"/>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A113" s="57"/>
       <c r="B113" s="64"/>
       <c r="C113" s="62"/>
@@ -4934,7 +4961,7 @@
       <c r="G113" s="37"/>
       <c r="H113" s="8"/>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A114" s="55"/>
       <c r="B114" s="64"/>
       <c r="C114" s="62"/>
@@ -4942,7 +4969,7 @@
       <c r="G114" s="37"/>
       <c r="H114" s="8"/>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A115" s="56"/>
       <c r="B115" s="64"/>
       <c r="C115" s="62"/>
@@ -4950,7 +4977,7 @@
       <c r="G115" s="37"/>
       <c r="H115" s="8"/>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A116" s="57"/>
       <c r="B116" s="64"/>
       <c r="C116" s="62"/>
@@ -4958,7 +4985,7 @@
       <c r="G116" s="37"/>
       <c r="H116" s="8"/>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A117" s="57"/>
       <c r="B117" s="64"/>
       <c r="C117" s="62"/>
@@ -4966,7 +4993,7 @@
       <c r="G117" s="37"/>
       <c r="H117" s="8"/>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A118" s="57"/>
       <c r="B118" s="64"/>
       <c r="C118" s="62"/>
@@ -4974,7 +5001,7 @@
       <c r="G118" s="37"/>
       <c r="H118" s="8"/>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A119" s="55"/>
       <c r="B119" s="64"/>
       <c r="C119" s="62"/>
@@ -4982,7 +5009,7 @@
       <c r="G119" s="37"/>
       <c r="H119" s="8"/>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A120" s="56"/>
       <c r="B120" s="64"/>
       <c r="C120" s="62"/>
@@ -4990,7 +5017,7 @@
       <c r="G120" s="37"/>
       <c r="H120" s="8"/>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A121" s="57"/>
       <c r="B121" s="64"/>
       <c r="C121" s="62"/>
@@ -4998,7 +5025,7 @@
       <c r="G121" s="37"/>
       <c r="H121" s="8"/>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A122" s="57"/>
       <c r="B122" s="64"/>
       <c r="C122" s="62"/>
@@ -5006,7 +5033,7 @@
       <c r="G122" s="37"/>
       <c r="H122" s="8"/>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A123" s="57"/>
       <c r="B123" s="64"/>
       <c r="C123" s="62"/>
@@ -5014,7 +5041,7 @@
       <c r="G123" s="37"/>
       <c r="H123" s="8"/>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A124" s="55"/>
       <c r="B124" s="64"/>
       <c r="C124" s="62"/>
@@ -5022,7 +5049,7 @@
       <c r="G124" s="37"/>
       <c r="H124" s="8"/>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A125" s="56"/>
       <c r="B125" s="64"/>
       <c r="C125" s="62"/>
@@ -5030,7 +5057,7 @@
       <c r="G125" s="37"/>
       <c r="H125" s="8"/>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A126" s="57"/>
       <c r="B126" s="64"/>
       <c r="C126" s="62"/>
@@ -5038,7 +5065,7 @@
       <c r="G126" s="37"/>
       <c r="H126" s="8"/>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A127" s="57"/>
       <c r="B127" s="64"/>
       <c r="C127" s="62"/>
@@ -5046,7 +5073,7 @@
       <c r="G127" s="37"/>
       <c r="H127" s="8"/>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A128" s="57"/>
       <c r="B128" s="64"/>
       <c r="C128" s="62"/>
@@ -5054,7 +5081,7 @@
       <c r="G128" s="37"/>
       <c r="H128" s="8"/>
     </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A129" s="55"/>
       <c r="B129" s="64"/>
       <c r="C129" s="62"/>
@@ -5062,7 +5089,7 @@
       <c r="G129" s="37"/>
       <c r="H129" s="8"/>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A130" s="56"/>
       <c r="B130" s="64"/>
       <c r="C130" s="62"/>
@@ -5070,7 +5097,7 @@
       <c r="G130" s="37"/>
       <c r="H130" s="8"/>
     </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A131" s="57"/>
       <c r="B131" s="64"/>
       <c r="C131" s="62"/>
@@ -5078,7 +5105,7 @@
       <c r="G131" s="37"/>
       <c r="H131" s="8"/>
     </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A132" s="57"/>
       <c r="B132" s="64"/>
       <c r="C132" s="62"/>
@@ -5086,7 +5113,7 @@
       <c r="G132" s="37"/>
       <c r="H132" s="8"/>
     </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A133" s="57"/>
       <c r="B133" s="64"/>
       <c r="C133" s="62"/>
@@ -5094,7 +5121,7 @@
       <c r="G133" s="37"/>
       <c r="H133" s="8"/>
     </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A134" s="55"/>
       <c r="B134" s="64"/>
       <c r="C134" s="62"/>
@@ -5102,7 +5129,7 @@
       <c r="G134" s="37"/>
       <c r="H134" s="8"/>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A135" s="56"/>
       <c r="B135" s="64"/>
       <c r="C135" s="62"/>
@@ -5110,7 +5137,7 @@
       <c r="G135" s="37"/>
       <c r="H135" s="8"/>
     </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A136" s="57"/>
       <c r="B136" s="64"/>
       <c r="C136" s="62"/>
@@ -5118,7 +5145,7 @@
       <c r="G136" s="37"/>
       <c r="H136" s="8"/>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A137" s="57"/>
       <c r="B137" s="64"/>
       <c r="C137" s="62"/>
@@ -5126,7 +5153,7 @@
       <c r="G137" s="37"/>
       <c r="H137" s="8"/>
     </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A138" s="57"/>
       <c r="B138" s="64"/>
       <c r="C138" s="62"/>
@@ -5134,7 +5161,7 @@
       <c r="G138" s="37"/>
       <c r="H138" s="8"/>
     </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A139" s="55"/>
       <c r="B139" s="64"/>
       <c r="C139" s="62"/>
@@ -5142,7 +5169,7 @@
       <c r="G139" s="37"/>
       <c r="H139" s="8"/>
     </row>
-    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A140" s="56"/>
       <c r="B140" s="64"/>
       <c r="C140" s="62"/>
@@ -5150,7 +5177,7 @@
       <c r="G140" s="37"/>
       <c r="H140" s="8"/>
     </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A141" s="57"/>
       <c r="B141" s="64"/>
       <c r="C141" s="62"/>
@@ -5158,7 +5185,7 @@
       <c r="G141" s="37"/>
       <c r="H141" s="8"/>
     </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A142" s="57"/>
       <c r="B142" s="64"/>
       <c r="C142" s="62"/>
@@ -5166,7 +5193,7 @@
       <c r="G142" s="37"/>
       <c r="H142" s="8"/>
     </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A143" s="57"/>
       <c r="B143" s="64"/>
       <c r="C143" s="62"/>
@@ -5174,7 +5201,7 @@
       <c r="G143" s="37"/>
       <c r="H143" s="8"/>
     </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A144" s="55"/>
       <c r="B144" s="64"/>
       <c r="C144" s="62"/>
@@ -5182,7 +5209,7 @@
       <c r="G144" s="37"/>
       <c r="H144" s="8"/>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A145" s="56"/>
       <c r="B145" s="64"/>
       <c r="C145" s="62"/>
@@ -5190,7 +5217,7 @@
       <c r="G145" s="37"/>
       <c r="H145" s="8"/>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A146" s="57"/>
       <c r="B146" s="64"/>
       <c r="C146" s="62"/>
@@ -5198,7 +5225,7 @@
       <c r="G146" s="37"/>
       <c r="H146" s="8"/>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A147" s="57"/>
       <c r="B147" s="64"/>
       <c r="C147" s="62"/>
@@ -5206,7 +5233,7 @@
       <c r="G147" s="37"/>
       <c r="H147" s="8"/>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A148" s="57"/>
       <c r="B148" s="64"/>
       <c r="C148" s="62"/>
@@ -5214,7 +5241,7 @@
       <c r="G148" s="37"/>
       <c r="H148" s="8"/>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A149" s="55"/>
       <c r="B149" s="64"/>
       <c r="C149" s="62"/>
@@ -5222,7 +5249,7 @@
       <c r="G149" s="37"/>
       <c r="H149" s="8"/>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A150" s="56"/>
       <c r="B150" s="64"/>
       <c r="C150" s="62"/>
@@ -5230,7 +5257,7 @@
       <c r="G150" s="37"/>
       <c r="H150" s="8"/>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A151" s="57"/>
       <c r="B151" s="64"/>
       <c r="C151" s="62"/>
@@ -5238,7 +5265,7 @@
       <c r="G151" s="37"/>
       <c r="H151" s="8"/>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A152" s="57"/>
       <c r="B152" s="64"/>
       <c r="C152" s="62"/>
@@ -5258,14 +5285,14 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5276,7 +5303,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -5287,7 +5314,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>0</v>
       </c>
@@ -5306,9 +5333,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C903B846-9155-4C37-ABE1-59FA4D45CD76}">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5316,22 +5343,22 @@
         <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -5342,10 +5369,10 @@
         <v>4</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>34</v>
@@ -5354,15 +5381,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="D3" s="3">
         <v>30.8</v>
@@ -5377,15 +5404,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="D4" s="3">
         <v>119</v>
@@ -5408,9 +5435,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{387AF5AC-D97C-4B95-B84B-AE3277E9ED2E}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5418,25 +5445,25 @@
         <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -5444,10 +5471,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>34</v>
@@ -5462,12 +5489,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="C3" s="4">
         <v>18308</v>

</xml_diff>